<commit_message>
refactor(schema): make the record base a mixin so adapt can root records
Signed-off-by: noelmcloughlin <noel.mcloughlin@gmail.com>
</commit_message>
<xml_diff>
--- a/project/excel/iso27001.xlsx
+++ b/project/excel/iso27001.xlsx
@@ -850,102 +850,102 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -1021,102 +1021,102 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="AD1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AE1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -1147,102 +1147,102 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -1631,102 +1631,102 @@
       </c>
       <c r="J1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AC1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -1863,102 +1863,102 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -1984,102 +1984,102 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -2156,102 +2156,102 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -2307,102 +2307,102 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -2428,102 +2428,102 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="S1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="T1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="U1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -2645,102 +2645,102 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -2836,102 +2836,102 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -3192,102 +3192,102 @@
       </c>
       <c r="P1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="AG1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="AH1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AI1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -3796,102 +3796,102 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="Y1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -3937,102 +3937,102 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="V1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="W1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="X1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -4255,102 +4255,102 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>
@@ -4411,102 +4411,102 @@
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>isms_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
           <t>document_reference</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>document_version</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>document_author</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>document_owner</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>document_approver</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>document_approval_date</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>document_effective_date</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>document_last_review_date</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>document_next_review_date</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>document_status</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>document_classification</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>document_retention</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>document_distribution</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>document_storage</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>document_change_control</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>document_external_origin</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>document_external_source</t>
-        </is>
-      </c>
-      <c r="Z1" t="inlineStr">
-        <is>
-          <t>isms_id</t>
-        </is>
-      </c>
-      <c r="AA1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="AB1" t="inlineStr">
-        <is>
-          <t>description</t>
         </is>
       </c>
     </row>

</xml_diff>